<commit_message>
Corregir logo (no encimar el titulo) y ensanchar columna SI/NO
Aplica los dos ajustes que indico el usuario:
- Logo: se reemplaza el dibujo de la plantilla base por la version con
  el anclaje corregido (imagen mas pequena y en la banda superior, sin
  encimarse con el titulo). La imagen es la misma; solo cambia la
  geometria del twoCellAnchor.
- Columna "(colocar SI o NO)": ancho 63 (antes 20) para que haya espacio
  de escribir; la columna MARCA queda en 50.

Cambios en las dos versiones (HTML/ExcelJS y Python/openpyxl) + rebuild
de docs/index.html. Verificado contra el archivo corregido del usuario:
valores, anclaje del logo, anchos y combinaciones coinciden.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S69ej8Vgbpjdhn84ABgydA
</commit_message>
<xml_diff>
--- a/plantilla/FORMATO_VALIDACIONES_DE_BIENES.xlsx
+++ b/plantilla/FORMATO_VALIDACIONES_DE_BIENES.xlsx
@@ -496,52 +496,43 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>228480</xdr:colOff>
+      <xdr:colOff>228481</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>190502</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>6715125</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>485775</xdr:rowOff>
+      <xdr:colOff>1854611</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1666875</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E84147F8-FF77-4661-BB50-9350BCAF74A7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="418980" y="723902"/>
-          <a:ext cx="14782920" cy="2181223"/>
+          <a:off x="418981" y="714377"/>
+          <a:ext cx="9912880" cy="1476373"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>

</xml_diff>